<commit_message>
impor mitra pake thaun
</commit_message>
<xml_diff>
--- a/public/templates/template_mitra.xlsx
+++ b/public/templates/template_mitra.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12180"/>
+    <workbookView windowWidth="14400" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="37">
   <si>
     <t>Nama Lengkap</t>
   </si>
@@ -87,6 +87,9 @@
   </si>
   <si>
     <t>Atas Nama</t>
+  </si>
+  <si>
+    <t>Tahun</t>
   </si>
   <si>
     <t>Contoh</t>
@@ -773,7 +776,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="49">
@@ -788,7 +791,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1166,7 +1169,9 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1"/>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
       <c r="V1" s="1"/>
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
@@ -1179,7 +1184,7 @@
       <c r="AE1" s="1"/>
       <c r="AF1" s="1"/>
     </row>
-    <row r="2" spans="1:32">
+    <row r="2" ht="15.75" spans="1:32">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1213,57 +1218,60 @@
       <c r="AE2" s="2"/>
       <c r="AF2" s="2"/>
     </row>
-    <row r="3" ht="15.75" spans="1:17">
+    <row r="3" spans="1:32">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
-        <v>21</v>
-      </c>
       <c r="E3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="M3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="N3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="P3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="Q3" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="U3">
+        <v>2028</v>
       </c>
     </row>
   </sheetData>

</xml_diff>